<commit_message>
Add readtable support for leading empty rows...
</commit_message>
<xml_diff>
--- a/data/EmptyTableRows.xlsx
+++ b/data/EmptyTableRows.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ee85442dac9ca7a7/Documents/Julia/XLSX/XLSX.jl/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{FD4869DF-CDF6-411F-98D7-9832212F3C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12E8ED91-BE29-48D5-8AFE-296EA46FB409}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="8_{FD4869DF-CDF6-411F-98D7-9832212F3C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF868A60-4002-4A3F-8D28-5781C3E3E616}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{D0B04E13-E96B-49ED-A7EE-BBA69F67C51D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{D0B04E13-E96B-49ED-A7EE-BBA69F67C51D}"/>
   </bookViews>
   <sheets>
     <sheet name="EmptyRow" sheetId="1" r:id="rId1"/>
     <sheet name="EmptyCols" sheetId="2" r:id="rId2"/>
     <sheet name="MixedEmpty" sheetId="3" r:id="rId3"/>
+    <sheet name="LeadingEmpty" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="9">
   <si>
     <t>Col B</t>
   </si>
@@ -59,6 +60,12 @@
   </si>
   <si>
     <t>Col A</t>
+  </si>
+  <si>
+    <t>col A</t>
+  </si>
+  <si>
+    <t>col B</t>
   </si>
 </sst>
 </file>
@@ -560,10 +567,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03E8D532-1601-4D72-BFF9-091E63B5F0F0}">
-  <dimension ref="A2:C32"/>
+  <dimension ref="A2:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>6</v>
       </c>
@@ -571,7 +578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>1</v>
       </c>
@@ -579,7 +586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>2</v>
       </c>
@@ -587,12 +594,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>3</v>
       </c>
@@ -600,7 +602,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>4</v>
       </c>
@@ -608,7 +610,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>5</v>
       </c>
@@ -616,17 +618,23 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B15">
         <v>6</v>
       </c>
@@ -634,7 +642,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B16">
         <v>7</v>
       </c>
@@ -642,7 +650,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B17">
         <v>8</v>
       </c>
@@ -650,22 +658,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B25">
         <v>9</v>
       </c>
@@ -673,7 +689,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B26">
         <v>10</v>
       </c>
@@ -681,7 +697,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B27">
         <v>11</v>
       </c>
@@ -689,7 +705,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B28">
         <v>12</v>
       </c>
@@ -697,7 +713,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B29">
         <v>13</v>
       </c>
@@ -705,7 +721,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B30">
         <v>14</v>
       </c>
@@ -713,7 +729,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B31">
         <v>15</v>
       </c>
@@ -721,11 +737,157 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B32">
         <v>16</v>
       </c>
       <c r="C32" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26D53932-19C4-4281-AAFA-BF2FC1FB8812}">
+  <dimension ref="B2:C35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>4</v>
+      </c>
+      <c r="C11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B12">
+        <v>5</v>
+      </c>
+      <c r="C12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <v>6</v>
+      </c>
+      <c r="C18" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19">
+        <v>7</v>
+      </c>
+      <c r="C19" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B28">
+        <v>9</v>
+      </c>
+      <c r="C28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B29">
+        <v>10</v>
+      </c>
+      <c r="C29" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B30">
+        <v>11</v>
+      </c>
+      <c r="C30" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B31">
+        <v>12</v>
+      </c>
+      <c r="C31" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B32">
+        <v>13</v>
+      </c>
+      <c r="C32" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B33">
+        <v>14</v>
+      </c>
+      <c r="C33" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B34">
+        <v>15</v>
+      </c>
+      <c r="C34" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B35">
+        <v>16</v>
+      </c>
+      <c r="C35" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
More fixes and tests for corner cases of #312
</commit_message>
<xml_diff>
--- a/data/EmptyTableRows.xlsx
+++ b/data/EmptyTableRows.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ee85442dac9ca7a7/Documents/Julia/XLSX/XLSX.jl/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="8_{FD4869DF-CDF6-411F-98D7-9832212F3C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF868A60-4002-4A3F-8D28-5781C3E3E616}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="8_{FD4869DF-CDF6-411F-98D7-9832212F3C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4148584-E561-45B1-A1DC-75897F5E718E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{D0B04E13-E96B-49ED-A7EE-BBA69F67C51D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{D0B04E13-E96B-49ED-A7EE-BBA69F67C51D}"/>
   </bookViews>
   <sheets>
     <sheet name="EmptyRow" sheetId="1" r:id="rId1"/>
     <sheet name="EmptyCols" sheetId="2" r:id="rId2"/>
     <sheet name="MixedEmpty" sheetId="3" r:id="rId3"/>
     <sheet name="LeadingEmpty" sheetId="4" r:id="rId4"/>
+    <sheet name="LeadingMixed" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="9">
   <si>
     <t>Col B</t>
   </si>
@@ -894,4 +895,160 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD1914AA-9191-489F-B71F-A482E6185745}">
+  <dimension ref="A2:C35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>4</v>
+      </c>
+      <c r="C11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B12">
+        <v>5</v>
+      </c>
+      <c r="C12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <v>6</v>
+      </c>
+      <c r="C18" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19">
+        <v>7</v>
+      </c>
+      <c r="C19" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B28">
+        <v>9</v>
+      </c>
+      <c r="C28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B29">
+        <v>10</v>
+      </c>
+      <c r="C29" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B30">
+        <v>11</v>
+      </c>
+      <c r="C30" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B31">
+        <v>12</v>
+      </c>
+      <c r="C31" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B32">
+        <v>13</v>
+      </c>
+      <c r="C32" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B33">
+        <v>14</v>
+      </c>
+      <c r="C33" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B34">
+        <v>15</v>
+      </c>
+      <c r="C34" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B35">
+        <v>16</v>
+      </c>
+      <c r="C35" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>